<commit_message>
Deployed a85435f with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/disciplines-revues.xlsx
+++ b/downloads/disciplines-revues.xlsx
@@ -544,7 +544,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arts</t>
+          <t>Littérature</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -557,7 +557,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Études des aires culturelles</t>
+          <t>Arts</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -570,7 +570,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Littérature</t>
+          <t>Sciences politiques</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -583,7 +583,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sciences politiques</t>
+          <t>Études des aires culturelles</t>
         </is>
       </c>
       <c r="B12" t="n">

</xml_diff>